<commit_message>
Quality audit complete: fixed dataset, SQL, EDA, and README
</commit_message>
<xml_diff>
--- a/excel/Cost_of_Quality_Analysis.xlsx
+++ b/excel/Cost_of_Quality_Analysis.xlsx
@@ -207,16 +207,16 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>325800</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>17376</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>27500</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>343176</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -616,7 +616,7 @@
         <v>8</v>
       </c>
       <c r="E4" s="4">
-        <v>0</v>
+        <v>325800</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -624,13 +624,13 @@
         <v>3</v>
       </c>
       <c r="B5" s="5">
-        <v>0.9608772727272727</v>
+        <v>0.9374377818181818</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E5" s="4">
-        <v>0</v>
+        <v>17376</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -638,7 +638,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="3">
-        <v>0</v>
+        <v>724</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>10</v>
@@ -658,7 +658,7 @@
         <v>11</v>
       </c>
       <c r="E7" s="4">
-        <v>0</v>
+        <v>343176</v>
       </c>
     </row>
   </sheetData>

</xml_diff>